<commit_message>
fix: validate generated test artifacts across commits
</commit_message>
<xml_diff>
--- a/features/RC-001-red-score/docs/v2/test-spec/test-case-report.xlsx
+++ b/features/RC-001-red-score/docs/v2/test-spec/test-case-report.xlsx
@@ -18797,7 +18797,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>v2 working tree based on fd0bc963c075cb4a8d6846bf210d1761344a1355; exact source hashes in manifest; pinned link pending commit</t>
+          <t>v2 working tree based on ffa72dc90f27fd128d62c5c092a5d3e8447a466a; exact source hashes in manifest; pinned link pending commit</t>
         </is>
       </c>
     </row>
@@ -54965,7 +54965,7 @@
   </sheetData>
   <autoFilter ref="A1:M570"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="0" sqref="D2:D570" showDropDown="0" showErrorMessage="1" errorStyle="stop">
+    <dataValidation showErrorMessage="1" type="list" allowBlank="0" sqref="D2:D570" errorStyle="stop" showDropDown="0">
       <formula1>"NOT RUN,PASS,FAIL,BLOCKED,SKIPPED"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>